<commit_message>
marketing: start Instagram plan on 2026-10-22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9SMZAeANtLs144Z5HZPdn
</commit_message>
<xml_diff>
--- a/marketing/instagram/tehvilaz-instagram.xlsx
+++ b/marketing/instagram/tehvilaz-instagram.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
marketing: start Instagram plan on 2026-10-22 (#29)
Claude-Session: https://claude.ai/code/session_01L9SMZAeANtLs144Z5HZPdn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/instagram/tehvilaz-instagram.xlsx
+++ b/marketing/instagram/tehvilaz-instagram.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">

</xml_diff>